<commit_message>
feat: accretion financing costs, target capex/NWC/minority inputs, EV from Uses, baseline FCF tests
- AccretionAnalysis: show financing costs (interest on new debt, preferred dividends) in accretion table
- DealReturnsMatrix: add target capex %, NWC %, and minority % input fields
- KeyMetricsCards: compute EV from Uses side, remove PF EV/EBITDA card
- helpers: add getEvFromUses utility
- dealReturns: add target_capex_pct_revenue, target_nwc_pct_revenue, minority_pct to DealParameters
- dealReturns.test: 446 lines of new baseline FCF computation tests
- i18n: add English and Norwegian keys for new UI fields
- types: extend DealParameters interface with new fields
</commit_message>
<xml_diff>
--- a/Div filer/Test Herjedal v2.xlsx
+++ b/Div filer/Test Herjedal v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pedrofasting/CODE/ECIT-acquisition/Div filer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{58EA7FF9-4238-554E-B050-AD14D4911139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551874D2-2B9D-FD48-B6C1-A7EFDD1CF605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{CD6F9456-AB92-5448-9CE2-F0C930A13991}"/>
   </bookViews>
@@ -102,9 +102,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0\ %"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000\ %"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -182,7 +183,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -199,6 +200,8 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -815,7 +818,7 @@
       <c r="A16" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="16">
         <v>0.01</v>
       </c>
       <c r="C16" s="15">
@@ -847,7 +850,7 @@
       <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="17">
         <f>C17/C9</f>
         <v>9.700176366843033E-3</v>
       </c>

</xml_diff>